<commit_message>
update excel import date protection
</commit_message>
<xml_diff>
--- a/static/format-upload/KAWI-import-selling-barge.xlsx
+++ b/static/format-upload/KAWI-import-selling-barge.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10824"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/meinardus/Project/python/mines-project/backend/static/format-upload/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/meinardus/Project/python/mines-project/backend/staticfiles/format-upload/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2123B561-4FE5-DE43-9AA6-A765C5D32FFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79C58E3C-A622-A14E-BD19-D34A4965D187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="880" windowWidth="36000" windowHeight="20100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -172,7 +172,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Date Dumoning DT ke Braging / Tongkang</t>
+          <t>Date Dumping DT ke Barging / Tongkang</t>
         </r>
       </text>
     </comment>
@@ -282,7 +282,16 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">Kode LOT :
-KWL- (LIM)
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">KWL- (LIM)
 </t>
         </r>
         <r>
@@ -325,7 +334,57 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>HPAL / RKEF</t>
+          <t xml:space="preserve">Untuk HPAL (LIM) / RKEF (SAP).
+</t>
+        </r>
+        <r>
+          <rPr>
+            <u/>
+            <sz val="8"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Note : 
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Original LIM dijual atau di blending jadi SAP maka diadjust jadi </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>RKEF</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">. Sebaliknya SAP ke LIM mejadi </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>HPAL</t>
         </r>
       </text>
     </comment>
@@ -483,7 +542,7 @@
     <numFmt numFmtId="165" formatCode="[$-409]d\-mmm\-yy;@"/>
     <numFmt numFmtId="166" formatCode="hh\.mm"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -538,6 +597,26 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="7">
@@ -687,7 +766,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -767,10 +846,7 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -1116,7 +1192,7 @@
     <col min="18" max="18" width="9" style="6" customWidth="1"/>
     <col min="19" max="19" width="12.5" style="6" customWidth="1"/>
     <col min="20" max="20" width="18.5" style="6" customWidth="1"/>
-    <col min="21" max="21" width="8.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.1640625" style="6" customWidth="1"/>
     <col min="22" max="22" width="12.1640625" style="6" customWidth="1"/>
     <col min="23" max="23" width="8.1640625" style="6" customWidth="1"/>
     <col min="24" max="24" width="12.1640625" style="6" customWidth="1"/>
@@ -1256,13 +1332,13 @@
         <f>X2</f>
         <v>1</v>
       </c>
-      <c r="S2" s="16" t="s">
+      <c r="S2" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="T2" s="12">
+      <c r="T2" s="28">
         <v>45873</v>
       </c>
-      <c r="U2" s="27"/>
+      <c r="U2" s="28"/>
       <c r="V2" s="24" t="str">
         <f>"SL_" &amp; TEXT(INT((COUNTIF($O$2:O2,O2)-1)/100)+1,"00")</f>
         <v>SL_01</v>
@@ -1299,9 +1375,9 @@
       <c r="P3" s="16"/>
       <c r="Q3" s="22"/>
       <c r="R3" s="16"/>
-      <c r="S3" s="16"/>
+      <c r="S3" s="27"/>
       <c r="T3" s="28"/>
-      <c r="U3" s="29"/>
+      <c r="U3" s="28"/>
       <c r="V3" s="24" t="str">
         <f>"SL_" &amp; TEXT(INT((COUNTIF($O$2:O3,O3)-1)/100)+1,"00")</f>
         <v>SL_00</v>
@@ -1338,9 +1414,9 @@
       <c r="P4" s="16"/>
       <c r="Q4" s="22"/>
       <c r="R4" s="16"/>
-      <c r="S4" s="16"/>
+      <c r="S4" s="27"/>
       <c r="T4" s="28"/>
-      <c r="U4" s="29"/>
+      <c r="U4" s="28"/>
       <c r="V4" s="24" t="str">
         <f>"SL_" &amp; TEXT(INT((COUNTIF($O$2:O4,O4)-1)/100)+1,"00")</f>
         <v>SL_00</v>
@@ -1377,9 +1453,9 @@
       <c r="P5" s="16"/>
       <c r="Q5" s="22"/>
       <c r="R5" s="16"/>
-      <c r="S5" s="16"/>
+      <c r="S5" s="27"/>
       <c r="T5" s="28"/>
-      <c r="U5" s="29"/>
+      <c r="U5" s="28"/>
       <c r="V5" s="24" t="str">
         <f>"SL_" &amp; TEXT(INT((COUNTIF($O$2:O5,O5)-1)/100)+1,"00")</f>
         <v>SL_00</v>
@@ -1416,9 +1492,9 @@
       <c r="P6" s="16"/>
       <c r="Q6" s="22"/>
       <c r="R6" s="16"/>
-      <c r="S6" s="16"/>
+      <c r="S6" s="27"/>
       <c r="T6" s="28"/>
-      <c r="U6" s="29"/>
+      <c r="U6" s="28"/>
       <c r="V6" s="24" t="str">
         <f>"SL_" &amp; TEXT(INT((COUNTIF($O$2:O6,O6)-1)/100)+1,"00")</f>
         <v>SL_00</v>
@@ -1455,9 +1531,9 @@
       <c r="P7" s="16"/>
       <c r="Q7" s="22"/>
       <c r="R7" s="16"/>
-      <c r="S7" s="16"/>
+      <c r="S7" s="27"/>
       <c r="T7" s="28"/>
-      <c r="U7" s="29"/>
+      <c r="U7" s="28"/>
       <c r="V7" s="24" t="str">
         <f>"SL_" &amp; TEXT(INT((COUNTIF($O$2:O7,O7)-1)/100)+1,"00")</f>
         <v>SL_00</v>

</xml_diff>